<commit_message>
sync v4.5.8: measurement appendix annotation cells cleared + 1A natural fluctuation
</commit_message>
<xml_diff>
--- a/results/measurement appendix.xlsx
+++ b/results/measurement appendix.xlsx
@@ -1613,31 +1613,31 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>618.7</v>
+        <v>597.2</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>191</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.946</v>
+        <v>0.951</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.054</v>
+        <v>0.052</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.046</v>
+        <v>0.043</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.054</v>
+        <v>0.057</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>19437.1</v>
+        <v>19414.6</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>90.3</v>
+        <v>68.8</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>4</v>
@@ -1660,31 +1660,31 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>657.3</v>
+        <v>643.9</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>191</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.931</v>
+        <v>0.929</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.049</v>
+        <v>0.051</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.057</v>
+        <v>0.052</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>19479.6</v>
+        <v>19465.3</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>128.9</v>
+        <v>115.5</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>4</v>
@@ -1707,31 +1707,31 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>812.2</v>
+        <v>786.4</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>195</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.916</v>
+        <v>0.918</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.902</v>
+        <v>0.903</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.066</v>
+        <v>0.064</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.057</v>
+        <v>0.054</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.065</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>19628.7</v>
+        <v>19601.8</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>283.8</v>
+        <v>258</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>8</v>
@@ -1754,31 +1754,31 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1024.5</v>
+        <v>1063.8</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>196</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.886</v>
+        <v>0.881</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.866</v>
+        <v>0.857</v>
       </c>
       <c r="H7" s="3" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="J7" s="3" t="n">
         <v>0.078</v>
       </c>
-      <c r="I7" s="3" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>0.082</v>
-      </c>
       <c r="K7" s="3" t="n">
-        <v>19836.3</v>
+        <v>19877.6</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>496.1</v>
+        <v>535.4</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>9</v>
@@ -1818,11 +1818,7 @@
       </c>
     </row>
     <row r="2" ht="59" customHeight="1" s="4">
-      <c r="A2" s="20" t="inlineStr">
-        <is>
-          <t>这里不是 MCFA，应该是普通 CFA！</t>
-        </is>
-      </c>
+      <c r="A2" s="20" t="n"/>
       <c r="L2" s="14" t="n"/>
       <c r="M2" s="14" t="n"/>
       <c r="N2" s="14" t="n"/>
@@ -2064,17 +2060,7 @@
       </c>
     </row>
     <row r="2" ht="248" customHeight="1" s="4">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>也是普通 CFA，不是 MCFA！
-要跑的模型是：
-Two-factor model：
-leader-rated OCBS
-leader-rated CWBS
-One-factor model：
-leader-rated OCBS 和 CWBS 合并</t>
-        </is>
-      </c>
+      <c r="A2" s="15" t="n"/>
       <c r="I2" s="14" t="n"/>
       <c r="J2" s="14" t="n"/>
       <c r="K2" s="14" t="n"/>
@@ -2232,17 +2218,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="208" customHeight="1" s="4">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>也是普通 CFA，不是 MCFA！
-要跑的模型是：
-Two-factor model：
-follower-rated OCBS
-follower-rated CWBS
-One-factor model：
-follower-rated OCBS 和 CWBS 合并</t>
-        </is>
-      </c>
+      <c r="A1" s="6" t="n"/>
     </row>
     <row r="2" ht="20.25" customHeight="1" s="4">
       <c r="A2" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(A1): split Thriving into T1+T3 rows in single-construct CFA table
Customer noted Table A1 was missing a row — needs both T1 and T3 Thriving
single-construct CFA. Inserted Thriving (T3) row; relabeled existing to
Thriving (T1). Both 10-item, MLR:
  Thriving (T1): CFI=0.985 RMSEA=0.063
  Thriving (T3): CFI=0.964 RMSEA=0.072
OCBS/CWBS rows shifted down; Table A2 leader-rated shifted to R17/18.
219/219 + 10/10 PASS.
</commit_message>
<xml_diff>
--- a/results/measurement appendix.xlsx
+++ b/results/measurement appendix.xlsx
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="33.375" customWidth="1" style="4" min="9" max="9"/>
@@ -2579,7 +2579,7 @@
     <row r="9" ht="15" customHeight="1" s="4">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Thriving</t>
+          <t>Thriving (T1)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -2605,170 +2605,198 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="4">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Self-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>6</v>
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Thriving (T3)</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>18.1</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>0.985</v>
+        <v>0.964</v>
       </c>
       <c r="F10" t="n">
-        <v>0.975</v>
+        <v>0.954</v>
       </c>
       <c r="G10" t="n">
-        <v>0.055</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.027</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" s="4">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Self-rated OCBS</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.027</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Self-rated CWBS</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>6.3</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>0.997</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F12" t="n">
         <v>0.995</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G12" t="n">
         <v>0.028</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H12" t="n">
         <v>0.018</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13"/>
-    <row r="14" ht="20.25" customHeight="1" s="4">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="14" ht="20.25" customHeight="1" s="4"/>
+    <row r="15" ht="28.5" customHeight="1" s="4">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Table A2 Single-Construct CFAs for Leader-Rated Behavioral Measures</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28.5" customHeight="1" s="4">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="45" customHeight="1" s="4">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Construct</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Items used</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>χ²</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>CFI</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>TLI</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>RMSEA</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>SRMR</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1" s="4">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Leader-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="D16" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.02</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" s="4">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Leader-rated OCBS</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D17" t="n">
+        <v>9</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Leader-rated CWBS</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B18" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C18" t="n">
         <v>5.4</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>5</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>0.999</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>0.999</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>0.014</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H18" t="n">
         <v>0.018</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(A1): Thriving T1+T3 rows (sync from main)
</commit_message>
<xml_diff>
--- a/results/measurement appendix.xlsx
+++ b/results/measurement appendix.xlsx
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="33.375" customWidth="1" style="4" min="9" max="9"/>
@@ -2579,7 +2579,7 @@
     <row r="9" ht="15" customHeight="1" s="4">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Thriving</t>
+          <t>Thriving (T1)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -2605,170 +2605,198 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="4">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Self-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>6</v>
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Thriving (T3)</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>18.1</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>0.985</v>
+        <v>0.964</v>
       </c>
       <c r="F10" t="n">
-        <v>0.975</v>
+        <v>0.954</v>
       </c>
       <c r="G10" t="n">
-        <v>0.055</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.027</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" s="4">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Self-rated OCBS</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.027</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Self-rated CWBS</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>6.3</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>0.997</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F12" t="n">
         <v>0.995</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G12" t="n">
         <v>0.028</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H12" t="n">
         <v>0.018</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13"/>
-    <row r="14" ht="20.25" customHeight="1" s="4">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="14" ht="20.25" customHeight="1" s="4"/>
+    <row r="15" ht="28.5" customHeight="1" s="4">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Table A2 Single-Construct CFAs for Leader-Rated Behavioral Measures</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28.5" customHeight="1" s="4">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="45" customHeight="1" s="4">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Construct</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Items used</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>χ²</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>CFI</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>TLI</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>RMSEA</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>SRMR</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1" s="4">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Leader-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="D16" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.02</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" s="4">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Leader-rated OCBS</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D17" t="n">
+        <v>9</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Leader-rated CWBS</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B18" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C18" t="n">
         <v>5.4</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>5</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>0.999</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>0.999</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>0.014</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H18" t="n">
         <v>0.018</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(A1): Thriving T1+T3 rows (Version B)
</commit_message>
<xml_diff>
--- a/results/measurement appendix.xlsx
+++ b/results/measurement appendix.xlsx
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="33.375" customWidth="1" style="4" min="9" max="9"/>
@@ -2579,7 +2579,7 @@
     <row r="9" ht="15" customHeight="1" s="4">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Thriving</t>
+          <t>Thriving (T1)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -2605,170 +2605,198 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="4">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Self-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>6</v>
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Thriving (T3)</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>31.4</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>0.951</v>
+        <v>0.964</v>
       </c>
       <c r="F10" t="n">
-        <v>0.918</v>
+        <v>0.954</v>
       </c>
       <c r="G10" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.04</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" s="4">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Self-rated OCBS</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.951</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Self-rated CWBS</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>11.1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>0.983</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F12" t="n">
         <v>0.965</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G12" t="n">
         <v>0.06</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H12" t="n">
         <v>0.028</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13"/>
-    <row r="14" ht="20.25" customHeight="1" s="4">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="14" ht="20.25" customHeight="1" s="4"/>
+    <row r="15" ht="28.5" customHeight="1" s="4">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Table A2 Single-Construct CFAs for Leader-Rated Behavioral Measures</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28.5" customHeight="1" s="4">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="45" customHeight="1" s="4">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Construct</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Items used</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>χ²</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>CFI</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>TLI</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>RMSEA</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>SRMR</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1" s="4">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Leader-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="D16" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1.005</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.02</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" s="4">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Leader-rated CWBS</t>
+          <t>Leader-rated OCBS</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>4.7</v>
+        <v>7.6</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1.002</v>
+        <v>1.005</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Leader-rated CWBS</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.002</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>0.018</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(A1): Thriving T1+T3 rows (Version B sync)
</commit_message>
<xml_diff>
--- a/results/measurement appendix.xlsx
+++ b/results/measurement appendix.xlsx
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="33.375" customWidth="1" style="4" min="9" max="9"/>
@@ -2579,7 +2579,7 @@
     <row r="9" ht="15" customHeight="1" s="4">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Thriving</t>
+          <t>Thriving (T1)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -2605,170 +2605,198 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="4">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Self-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>6</v>
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Thriving (T3)</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>31.4</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>0.951</v>
+        <v>0.964</v>
       </c>
       <c r="F10" t="n">
-        <v>0.918</v>
+        <v>0.954</v>
       </c>
       <c r="G10" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.04</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" s="4">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Self-rated OCBS</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.951</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Self-rated CWBS</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>11.1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>0.983</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F12" t="n">
         <v>0.965</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G12" t="n">
         <v>0.06</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H12" t="n">
         <v>0.028</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13"/>
-    <row r="14" ht="20.25" customHeight="1" s="4">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="14" ht="20.25" customHeight="1" s="4"/>
+    <row r="15" ht="28.5" customHeight="1" s="4">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Table A2 Single-Construct CFAs for Leader-Rated Behavioral Measures</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28.5" customHeight="1" s="4">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="45" customHeight="1" s="4">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Construct</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Items used</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>χ²</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>CFI</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>TLI</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>RMSEA</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>SRMR</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1" s="4">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Leader-rated OCBS</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="D16" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1.005</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.02</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" s="4">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Leader-rated CWBS</t>
+          <t>Leader-rated OCBS</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>4.7</v>
+        <v>7.6</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1.002</v>
+        <v>1.005</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Leader-rated CWBS</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.002</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>0.018</v>
       </c>
     </row>

</xml_diff>